<commit_message>
Add PiN step 1 hybrid for Somalia___SOM
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Somalia___SOM/PiN_step1_Somalia___SOM_1022_12PM.xlsx
+++ b/platform_PiN_output/Somalia___SOM/PiN_step1_Somalia___SOM_1022_12PM.xlsx
@@ -1747,37 +1747,37 @@
         </is>
       </c>
       <c r="C5" s="33" t="n">
-        <v>15</v>
+        <v>17086</v>
       </c>
       <c r="D5" s="33" t="n">
-        <v>34.3</v>
+        <v>40.8</v>
       </c>
       <c r="E5" s="33" t="n">
-        <v>5</v>
+        <v>6978</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>61.3</v>
+        <v>53.5</v>
       </c>
       <c r="G5" s="33" t="n">
-        <v>9</v>
+        <v>9146</v>
       </c>
       <c r="H5" s="33" t="n">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="I5" s="33" t="n">
-        <v>1</v>
+        <v>722</v>
       </c>
       <c r="J5" s="33" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="K5" s="33" t="n">
-        <v>0</v>
+        <v>241</v>
       </c>
       <c r="L5" s="33" t="n">
-        <v>65.7</v>
+        <v>59.2</v>
       </c>
       <c r="M5" s="33" t="n">
-        <v>10</v>
+        <v>10108</v>
       </c>
       <c r="N5" s="34" t="inlineStr">
         <is>
@@ -1994,7 +1994,7 @@
         <v>0</v>
       </c>
       <c r="CD5" s="49" t="n">
-        <v>1.011302003253337</v>
+        <v>0.0008878339019548199</v>
       </c>
     </row>
     <row r="6">
@@ -2009,40 +2009,42 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v/>
+        <v>15492</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v/>
+        <v>37.8</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v/>
+        <v>5850</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v/>
+        <v>55.2</v>
       </c>
       <c r="G6" s="33" t="n">
-        <v/>
+        <v>8558</v>
       </c>
       <c r="H6" s="33" t="n">
-        <v/>
+        <v>7</v>
       </c>
       <c r="I6" s="33" t="n">
-        <v/>
+        <v>1083</v>
       </c>
       <c r="J6" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K6" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="L6" s="33" t="n">
-        <v/>
+        <v>62.2</v>
       </c>
       <c r="M6" s="33" t="n">
-        <v/>
-      </c>
-      <c r="N6" s="34" t="n">
-        <v/>
+        <v>9642</v>
+      </c>
+      <c r="N6" s="34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="O6" s="35" t="n">
         <v/>
@@ -2253,10 +2255,8 @@
       <c r="CC6" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="CD6" s="49" t="inlineStr">
-        <is>
-          <t>&lt;NA&gt;</t>
-        </is>
+      <c r="CD6" s="49" t="n">
+        <v>0.002169985344030699</v>
       </c>
     </row>
     <row r="7">
@@ -2553,41 +2553,41 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>0</v>
+        <v>36044</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v/>
+        <v>82.8</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>0</v>
+        <v>29828</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v/>
+        <v>15.7</v>
       </c>
       <c r="G8" s="33" t="n">
-        <v>0</v>
+        <v>5652</v>
       </c>
       <c r="H8" s="33" t="n">
-        <v/>
+        <v>1.2</v>
       </c>
       <c r="I8" s="33" t="n">
-        <v>0</v>
+        <v>440</v>
       </c>
       <c r="J8" s="33" t="n">
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="K8" s="33" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="L8" s="33" t="n">
-        <v/>
+        <v>17.2</v>
       </c>
       <c r="M8" s="33" t="n">
-        <v>0</v>
+        <v>6217</v>
       </c>
       <c r="N8" s="34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="O8" s="35" t="n">
@@ -2815,40 +2815,42 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v/>
+        <v>23365</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v/>
+        <v>42.9</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v/>
+        <v>10027</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v/>
+        <v>47.2</v>
       </c>
       <c r="G9" s="33" t="n">
-        <v/>
+        <v>11039</v>
       </c>
       <c r="H9" s="33" t="n">
-        <v/>
+        <v>9.800000000000001</v>
       </c>
       <c r="I9" s="33" t="n">
-        <v/>
+        <v>2300</v>
       </c>
       <c r="J9" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K9" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="L9" s="33" t="n">
-        <v/>
+        <v>57.1</v>
       </c>
       <c r="M9" s="33" t="n">
-        <v/>
-      </c>
-      <c r="N9" s="34" t="n">
-        <v/>
+        <v>13339</v>
+      </c>
+      <c r="N9" s="34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="O9" s="35" t="n">
         <v/>
@@ -3059,10 +3061,8 @@
       <c r="CC9" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="CD9" s="49" t="inlineStr">
-        <is>
-          <t>&lt;NA&gt;</t>
-        </is>
+      <c r="CD9" s="49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -3339,37 +3339,37 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>5944</v>
+        <v>37338</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>37.9</v>
+        <v>41.2</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>2255</v>
+        <v>15383</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>54.3</v>
+        <v>55.2</v>
       </c>
       <c r="G11" s="33" t="n">
-        <v>3228</v>
+        <v>20597</v>
       </c>
       <c r="H11" s="33" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="I11" s="33" t="n">
-        <v>102</v>
+        <v>755</v>
       </c>
       <c r="J11" s="33" t="n">
-        <v>6</v>
+        <v>1.6</v>
       </c>
       <c r="K11" s="33" t="n">
-        <v>359</v>
+        <v>603</v>
       </c>
       <c r="L11" s="33" t="n">
-        <v>62.1</v>
+        <v>58.8</v>
       </c>
       <c r="M11" s="33" t="n">
-        <v>3689</v>
+        <v>21955</v>
       </c>
       <c r="N11" s="34" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         <v>0</v>
       </c>
       <c r="CD11" s="49" t="n">
-        <v>1.00002227289775</v>
+        <v>0.1591979321362748</v>
       </c>
     </row>
     <row r="12">
@@ -3863,40 +3863,42 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v/>
+        <v>32784</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v/>
+        <v>25.4</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v/>
+        <v>8323</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v/>
+        <v>73.09999999999999</v>
       </c>
       <c r="G13" s="33" t="n">
-        <v/>
+        <v>23951</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v/>
+        <v>1.6</v>
       </c>
       <c r="I13" s="33" t="n">
-        <v/>
+        <v>510</v>
       </c>
       <c r="J13" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K13" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="L13" s="33" t="n">
-        <v/>
+        <v>74.59999999999999</v>
       </c>
       <c r="M13" s="33" t="n">
-        <v/>
-      </c>
-      <c r="N13" s="34" t="n">
-        <v/>
+        <v>24461</v>
+      </c>
+      <c r="N13" s="34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="O13" s="35" t="n">
         <v/>
@@ -4107,10 +4109,8 @@
       <c r="CC13" s="48" t="n">
         <v>0.04246723815154203</v>
       </c>
-      <c r="CD13" s="49" t="inlineStr">
-        <is>
-          <t>&lt;NA&gt;</t>
-        </is>
+      <c r="CD13" s="49" t="n">
+        <v>0.01289245669519038</v>
       </c>
     </row>
     <row r="14">
@@ -4911,40 +4911,42 @@
         </is>
       </c>
       <c r="C17" s="33" t="n">
-        <v/>
+        <v>9184</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v/>
+        <v>44</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v/>
+        <v>4039</v>
       </c>
       <c r="F17" s="33" t="n">
-        <v/>
+        <v>48.2</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v/>
+        <v>4426</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v/>
+        <v>7.8</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v/>
+        <v>719</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K17" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="L17" s="33" t="n">
-        <v/>
+        <v>56</v>
       </c>
       <c r="M17" s="33" t="n">
-        <v/>
-      </c>
-      <c r="N17" s="34" t="n">
-        <v/>
+        <v>5145</v>
+      </c>
+      <c r="N17" s="34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="O17" s="35" t="n">
         <v/>
@@ -5155,10 +5157,8 @@
       <c r="CC17" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="CD17" s="49" t="inlineStr">
-        <is>
-          <t>&lt;NA&gt;</t>
-        </is>
+      <c r="CD17" s="49" t="n">
+        <v>0.2654402195961406</v>
       </c>
     </row>
     <row r="18">
@@ -5743,37 +5743,37 @@
         </is>
       </c>
       <c r="C20" s="33" t="n">
-        <v>3884</v>
+        <v>65054</v>
       </c>
       <c r="D20" s="33" t="n">
-        <v>22.1</v>
+        <v>51.8</v>
       </c>
       <c r="E20" s="33" t="n">
-        <v>857</v>
+        <v>33724</v>
       </c>
       <c r="F20" s="33" t="n">
-        <v>76.5</v>
+        <v>47.1</v>
       </c>
       <c r="G20" s="33" t="n">
-        <v>2970</v>
+        <v>30664</v>
       </c>
       <c r="H20" s="33" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="I20" s="33" t="n">
         <v>29</v>
       </c>
       <c r="J20" s="33" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="K20" s="33" t="n">
-        <v>29</v>
+        <v>637</v>
       </c>
       <c r="L20" s="33" t="n">
-        <v>77.90000000000001</v>
+        <v>48.2</v>
       </c>
       <c r="M20" s="33" t="n">
-        <v>3027</v>
+        <v>31330</v>
       </c>
       <c r="N20" s="34" t="inlineStr">
         <is>
@@ -5990,7 +5990,7 @@
         <v>0.3987382515771855</v>
       </c>
       <c r="CD20" s="49" t="n">
-        <v>1.00000173853366</v>
+        <v>0.05970434950141016</v>
       </c>
     </row>
     <row r="21">
@@ -6267,37 +6267,37 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>11678</v>
+        <v>194353</v>
       </c>
       <c r="D22" s="33" t="n">
-        <v>22.3</v>
+        <v>48.9</v>
       </c>
       <c r="E22" s="33" t="n">
-        <v>2608</v>
+        <v>95083</v>
       </c>
       <c r="F22" s="33" t="n">
-        <v>63.6</v>
+        <v>42.4</v>
       </c>
       <c r="G22" s="33" t="n">
-        <v>7424</v>
+        <v>82465</v>
       </c>
       <c r="H22" s="33" t="n">
-        <v>8.9</v>
+        <v>3.7</v>
       </c>
       <c r="I22" s="33" t="n">
-        <v>1043</v>
+        <v>7107</v>
       </c>
       <c r="J22" s="33" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="K22" s="33" t="n">
-        <v>602</v>
+        <v>9698</v>
       </c>
       <c r="L22" s="33" t="n">
-        <v>77.7</v>
+        <v>51.1</v>
       </c>
       <c r="M22" s="33" t="n">
-        <v>9070</v>
+        <v>99270</v>
       </c>
       <c r="N22" s="34" t="inlineStr">
         <is>
@@ -6514,7 +6514,7 @@
         <v>0.250577867227762</v>
       </c>
       <c r="CD22" s="49" t="n">
-        <v>1.000000273150246</v>
+        <v>0.06008655996999569</v>
       </c>
     </row>
     <row r="23">
@@ -6529,37 +6529,37 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>1518</v>
+        <v>37221</v>
       </c>
       <c r="D23" s="33" t="n">
-        <v>49.2</v>
+        <v>69.7</v>
       </c>
       <c r="E23" s="33" t="n">
-        <v>746</v>
+        <v>25959</v>
       </c>
       <c r="F23" s="33" t="n">
-        <v>44.2</v>
+        <v>29</v>
       </c>
       <c r="G23" s="33" t="n">
-        <v>670</v>
+        <v>10808</v>
       </c>
       <c r="H23" s="33" t="n">
-        <v>5.4</v>
+        <v>1.2</v>
       </c>
       <c r="I23" s="33" t="n">
-        <v>82</v>
+        <v>435</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>1.3</v>
+        <v>0.1</v>
       </c>
       <c r="K23" s="33" t="n">
         <v>19</v>
       </c>
       <c r="L23" s="33" t="n">
-        <v>50.8</v>
+        <v>30.3</v>
       </c>
       <c r="M23" s="33" t="n">
-        <v>772</v>
+        <v>11262</v>
       </c>
       <c r="N23" s="34" t="inlineStr">
         <is>
@@ -6776,7 +6776,7 @@
         <v>0.05927210589405494</v>
       </c>
       <c r="CD23" s="49" t="n">
-        <v>1.000046668536021</v>
+        <v>0.04078533201251124</v>
       </c>
     </row>
     <row r="24">
@@ -6791,25 +6791,25 @@
         </is>
       </c>
       <c r="C24" s="33" t="n">
-        <v>63</v>
+        <v>46927</v>
       </c>
       <c r="D24" s="33" t="n">
-        <v>44.9</v>
+        <v>35.3</v>
       </c>
       <c r="E24" s="33" t="n">
-        <v>28</v>
+        <v>16569</v>
       </c>
       <c r="F24" s="33" t="n">
-        <v>54.5</v>
+        <v>62.9</v>
       </c>
       <c r="G24" s="33" t="n">
-        <v>34</v>
+        <v>29531</v>
       </c>
       <c r="H24" s="33" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="I24" s="33" t="n">
-        <v>0</v>
+        <v>827</v>
       </c>
       <c r="J24" s="33" t="n">
         <v>0</v>
@@ -6818,10 +6818,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="33" t="n">
-        <v>55.1</v>
+        <v>64.7</v>
       </c>
       <c r="M24" s="33" t="n">
-        <v>35</v>
+        <v>30359</v>
       </c>
       <c r="N24" s="34" t="inlineStr">
         <is>
@@ -7038,7 +7038,7 @@
         <v>0.007557292113224649</v>
       </c>
       <c r="CD24" s="49" t="n">
-        <v>1.003107799179588</v>
+        <v>0.001346682961798411</v>
       </c>
     </row>
     <row r="25">
@@ -7315,25 +7315,25 @@
         </is>
       </c>
       <c r="C26" s="33" t="n">
-        <v>490</v>
+        <v>64552</v>
       </c>
       <c r="D26" s="33" t="n">
-        <v>43.9</v>
+        <v>25.4</v>
       </c>
       <c r="E26" s="33" t="n">
-        <v>215</v>
+        <v>16375</v>
       </c>
       <c r="F26" s="33" t="n">
-        <v>50.5</v>
+        <v>60</v>
       </c>
       <c r="G26" s="33" t="n">
-        <v>247</v>
+        <v>38723</v>
       </c>
       <c r="H26" s="33" t="n">
-        <v>5.6</v>
+        <v>14.6</v>
       </c>
       <c r="I26" s="33" t="n">
-        <v>27</v>
+        <v>9454</v>
       </c>
       <c r="J26" s="33" t="n">
         <v>0</v>
@@ -7342,10 +7342,10 @@
         <v>0</v>
       </c>
       <c r="L26" s="33" t="n">
-        <v>56.1</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="M26" s="33" t="n">
-        <v>275</v>
+        <v>48177</v>
       </c>
       <c r="N26" s="34" t="inlineStr">
         <is>
@@ -7582,7 +7582,7 @@
         <v>0.1772293886707796</v>
       </c>
       <c r="CD26" s="49" t="n">
-        <v>0.9990911378539603</v>
+        <v>0.007583880554412575</v>
       </c>
     </row>
     <row r="27">
@@ -7597,37 +7597,37 @@
         </is>
       </c>
       <c r="C27" s="33" t="n">
-        <v>1505</v>
+        <v>51869</v>
       </c>
       <c r="D27" s="33" t="n">
-        <v>40.4</v>
+        <v>45.6</v>
       </c>
       <c r="E27" s="33" t="n">
-        <v>607</v>
+        <v>23661</v>
       </c>
       <c r="F27" s="33" t="n">
-        <v>56.7</v>
+        <v>51.9</v>
       </c>
       <c r="G27" s="33" t="n">
-        <v>854</v>
+        <v>26922</v>
       </c>
       <c r="H27" s="33" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="I27" s="33" t="n">
-        <v>38</v>
+        <v>1102</v>
       </c>
       <c r="J27" s="33" t="n">
         <v>0.4</v>
       </c>
       <c r="K27" s="33" t="n">
-        <v>5</v>
+        <v>183</v>
       </c>
       <c r="L27" s="33" t="n">
-        <v>59.6</v>
+        <v>54.4</v>
       </c>
       <c r="M27" s="33" t="n">
-        <v>897</v>
+        <v>28207</v>
       </c>
       <c r="N27" s="34" t="inlineStr">
         <is>
@@ -7844,7 +7844,7 @@
         <v>0.2060008032913234</v>
       </c>
       <c r="CD27" s="49" t="n">
-        <v>0.9999298646738988</v>
+        <v>0.02901336918649324</v>
       </c>
     </row>
     <row r="28">
@@ -7859,37 +7859,37 @@
         </is>
       </c>
       <c r="C28" s="33" t="n">
-        <v>187</v>
+        <v>34292</v>
       </c>
       <c r="D28" s="33" t="n">
-        <v>48.3</v>
+        <v>35.9</v>
       </c>
       <c r="E28" s="33" t="n">
-        <v>90</v>
+        <v>12321</v>
       </c>
       <c r="F28" s="33" t="n">
-        <v>49.5</v>
+        <v>62.2</v>
       </c>
       <c r="G28" s="33" t="n">
-        <v>92</v>
+        <v>21340</v>
       </c>
       <c r="H28" s="33" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="I28" s="33" t="n">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="J28" s="33" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="K28" s="33" t="n">
-        <v>4</v>
+        <v>474</v>
       </c>
       <c r="L28" s="33" t="n">
-        <v>51.7</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="M28" s="33" t="n">
-        <v>96</v>
+        <v>21971</v>
       </c>
       <c r="N28" s="34" t="inlineStr">
         <is>
@@ -8106,7 +8106,7 @@
         <v>0.0571134109159617</v>
       </c>
       <c r="CD28" s="49" t="n">
-        <v>0.9980582759867503</v>
+        <v>0.005442578374242456</v>
       </c>
     </row>
     <row r="29">
@@ -8737,37 +8737,37 @@
         </is>
       </c>
       <c r="C31" s="33" t="n">
-        <v>19148</v>
+        <v>67859</v>
       </c>
       <c r="D31" s="33" t="n">
-        <v>17.9</v>
+        <v>30.4</v>
       </c>
       <c r="E31" s="33" t="n">
-        <v>3435</v>
+        <v>20642</v>
       </c>
       <c r="F31" s="33" t="n">
-        <v>79.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="G31" s="33" t="n">
-        <v>15198</v>
+        <v>45690</v>
       </c>
       <c r="H31" s="33" t="n">
-        <v>2.7</v>
+        <v>2.1</v>
       </c>
       <c r="I31" s="33" t="n">
-        <v>515</v>
+        <v>1401</v>
       </c>
       <c r="J31" s="33" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K31" s="33" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="L31" s="33" t="n">
-        <v>82.09999999999999</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="M31" s="33" t="n">
-        <v>15713</v>
+        <v>47217</v>
       </c>
       <c r="N31" s="34" t="inlineStr">
         <is>
@@ -9004,7 +9004,7 @@
         <v>0.2448316924908958</v>
       </c>
       <c r="CD31" s="49" t="n">
-        <v>0.9999929712811214</v>
+        <v>0.2821713466760623</v>
       </c>
     </row>
     <row r="32">
@@ -9019,37 +9019,37 @@
         </is>
       </c>
       <c r="C32" s="33" t="n">
-        <v>5466</v>
+        <v>16974</v>
       </c>
       <c r="D32" s="33" t="n">
-        <v>23.1</v>
+        <v>10.3</v>
       </c>
       <c r="E32" s="33" t="n">
-        <v>1261</v>
+        <v>1741</v>
       </c>
       <c r="F32" s="33" t="n">
-        <v>74.40000000000001</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="G32" s="33" t="n">
-        <v>4064</v>
+        <v>13654</v>
       </c>
       <c r="H32" s="33" t="n">
-        <v>1.3</v>
+        <v>7.6</v>
       </c>
       <c r="I32" s="33" t="n">
-        <v>70</v>
+        <v>1295</v>
       </c>
       <c r="J32" s="33" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="K32" s="33" t="n">
-        <v>70</v>
+        <v>283</v>
       </c>
       <c r="L32" s="33" t="n">
-        <v>76.90000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="M32" s="33" t="n">
-        <v>4204</v>
+        <v>15233</v>
       </c>
       <c r="N32" s="34" t="inlineStr">
         <is>
@@ -9266,7 +9266,7 @@
         <v>0.05997768882472603</v>
       </c>
       <c r="CD32" s="49" t="n">
-        <v>0.9999324904603595</v>
+        <v>0.322000176320038</v>
       </c>
     </row>
     <row r="33">
@@ -9281,37 +9281,37 @@
         </is>
       </c>
       <c r="C33" s="33" t="n">
-        <v>383</v>
+        <v>10921</v>
       </c>
       <c r="D33" s="33" t="n">
-        <v>0.9</v>
+        <v>44.8</v>
       </c>
       <c r="E33" s="33" t="n">
-        <v>3</v>
+        <v>4889</v>
       </c>
       <c r="F33" s="33" t="n">
-        <v>93.8</v>
+        <v>53.1</v>
       </c>
       <c r="G33" s="33" t="n">
-        <v>359</v>
+        <v>5803</v>
       </c>
       <c r="H33" s="33" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="I33" s="33" t="n">
-        <v>14</v>
+        <v>223</v>
       </c>
       <c r="J33" s="33" t="n">
-        <v>1.8</v>
+        <v>0.1</v>
       </c>
       <c r="K33" s="33" t="n">
         <v>7</v>
       </c>
       <c r="L33" s="33" t="n">
-        <v>99.09999999999999</v>
+        <v>55.2</v>
       </c>
       <c r="M33" s="33" t="n">
-        <v>379</v>
+        <v>6032</v>
       </c>
       <c r="N33" s="34" t="inlineStr">
         <is>
@@ -9528,7 +9528,7 @@
         <v>0.3511450381679389</v>
       </c>
       <c r="CD33" s="49" t="n">
-        <v>0.9990650348292279</v>
+        <v>0.0350372592564412</v>
       </c>
     </row>
     <row r="34">
@@ -9543,37 +9543,37 @@
         </is>
       </c>
       <c r="C34" s="33" t="n">
-        <v>23519</v>
+        <v>57048</v>
       </c>
       <c r="D34" s="33" t="n">
-        <v>1.4</v>
+        <v>3.6</v>
       </c>
       <c r="E34" s="33" t="n">
-        <v>324</v>
+        <v>2057</v>
       </c>
       <c r="F34" s="33" t="n">
-        <v>93.09999999999999</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G34" s="33" t="n">
-        <v>21897</v>
+        <v>51590</v>
       </c>
       <c r="H34" s="33" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="I34" s="33" t="n">
-        <v>1216</v>
+        <v>2825</v>
       </c>
       <c r="J34" s="33" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="K34" s="33" t="n">
-        <v>81</v>
+        <v>576</v>
       </c>
       <c r="L34" s="33" t="n">
-        <v>98.59999999999999</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="M34" s="33" t="n">
-        <v>23194</v>
+        <v>54991</v>
       </c>
       <c r="N34" s="34" t="inlineStr">
         <is>
@@ -9790,7 +9790,7 @@
         <v>0.09863932614247056</v>
       </c>
       <c r="CD34" s="49" t="n">
-        <v>0.9999807650099746</v>
+        <v>0.4122589330435701</v>
       </c>
     </row>
     <row r="35">
@@ -10611,41 +10611,41 @@
         </is>
       </c>
       <c r="C38" s="33" t="n">
-        <v>0</v>
+        <v>247922</v>
       </c>
       <c r="D38" s="33" t="n">
-        <v/>
+        <v>31.4</v>
       </c>
       <c r="E38" s="33" t="n">
-        <v>0</v>
+        <v>77895</v>
       </c>
       <c r="F38" s="33" t="n">
-        <v/>
+        <v>68.2</v>
       </c>
       <c r="G38" s="33" t="n">
-        <v>0</v>
+        <v>169190</v>
       </c>
       <c r="H38" s="33" t="n">
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="I38" s="33" t="n">
-        <v>0</v>
+        <v>838</v>
       </c>
       <c r="J38" s="33" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="K38" s="33" t="n">
         <v>0</v>
       </c>
       <c r="L38" s="33" t="n">
-        <v/>
+        <v>68.59999999999999</v>
       </c>
       <c r="M38" s="33" t="n">
-        <v>0</v>
+        <v>170028</v>
       </c>
       <c r="N38" s="34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O38" s="35" t="n">
@@ -10863,41 +10863,41 @@
         </is>
       </c>
       <c r="C39" s="33" t="n">
-        <v>0</v>
+        <v>171981</v>
       </c>
       <c r="D39" s="33" t="n">
-        <v/>
+        <v>35.8</v>
       </c>
       <c r="E39" s="33" t="n">
-        <v>0</v>
+        <v>61588</v>
       </c>
       <c r="F39" s="33" t="n">
-        <v/>
+        <v>59.8</v>
       </c>
       <c r="G39" s="33" t="n">
-        <v>0</v>
+        <v>102840</v>
       </c>
       <c r="H39" s="33" t="n">
-        <v/>
+        <v>3.7</v>
       </c>
       <c r="I39" s="33" t="n">
-        <v>0</v>
+        <v>6391</v>
       </c>
       <c r="J39" s="33" t="n">
-        <v/>
+        <v>0.7</v>
       </c>
       <c r="K39" s="33" t="n">
-        <v>0</v>
+        <v>1162</v>
       </c>
       <c r="L39" s="33" t="n">
-        <v/>
+        <v>64.2</v>
       </c>
       <c r="M39" s="33" t="n">
-        <v>0</v>
+        <v>110393</v>
       </c>
       <c r="N39" s="34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O39" s="35" t="n">
@@ -11115,37 +11115,37 @@
         </is>
       </c>
       <c r="C40" s="33" t="n">
-        <v>43</v>
+        <v>60255</v>
       </c>
       <c r="D40" s="33" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="E40" s="33" t="n">
-        <v>0</v>
+        <v>36775</v>
       </c>
       <c r="F40" s="33" t="n">
-        <v>100</v>
+        <v>38.3</v>
       </c>
       <c r="G40" s="33" t="n">
-        <v>43</v>
+        <v>23099</v>
       </c>
       <c r="H40" s="33" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I40" s="33" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="J40" s="33" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="K40" s="33" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="L40" s="33" t="n">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="M40" s="33" t="n">
-        <v>43</v>
+        <v>23480</v>
       </c>
       <c r="N40" s="34" t="inlineStr">
         <is>
@@ -11382,7 +11382,7 @@
         <v>0.0697064546146688</v>
       </c>
       <c r="CD40" s="49" t="n">
-        <v>0.9915415578264181</v>
+        <v>0.0007075974937604511</v>
       </c>
     </row>
     <row r="41">
@@ -11397,37 +11397,37 @@
         </is>
       </c>
       <c r="C41" s="33" t="n">
-        <v>6247</v>
+        <v>74165</v>
       </c>
       <c r="D41" s="33" t="n">
-        <v>1.4</v>
+        <v>13.9</v>
       </c>
       <c r="E41" s="33" t="n">
-        <v>90</v>
+        <v>10342</v>
       </c>
       <c r="F41" s="33" t="n">
-        <v>97.09999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="G41" s="33" t="n">
-        <v>6067</v>
+        <v>62131</v>
       </c>
       <c r="H41" s="33" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="I41" s="33" t="n">
-        <v>90</v>
+        <v>411</v>
       </c>
       <c r="J41" s="33" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="K41" s="33" t="n">
-        <v>0</v>
+        <v>1281</v>
       </c>
       <c r="L41" s="33" t="n">
-        <v>98.59999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="M41" s="33" t="n">
-        <v>6157</v>
+        <v>63823</v>
       </c>
       <c r="N41" s="34" t="inlineStr">
         <is>
@@ -11680,7 +11680,7 @@
         <v>0.09919296044488904</v>
       </c>
       <c r="CD41" s="49" t="n">
-        <v>1.000013398355938</v>
+        <v>0.0842322348753394</v>
       </c>
     </row>
     <row r="42">
@@ -13097,37 +13097,37 @@
         </is>
       </c>
       <c r="C47" s="33" t="n">
-        <v>19897</v>
+        <v>176201</v>
       </c>
       <c r="D47" s="33" t="n">
-        <v>24.7</v>
+        <v>35.7</v>
       </c>
       <c r="E47" s="33" t="n">
-        <v>4923</v>
+        <v>62979</v>
       </c>
       <c r="F47" s="33" t="n">
-        <v>72.7</v>
+        <v>59.5</v>
       </c>
       <c r="G47" s="33" t="n">
-        <v>14461</v>
+        <v>104894</v>
       </c>
       <c r="H47" s="33" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="I47" s="33" t="n">
-        <v>513</v>
+        <v>6095</v>
       </c>
       <c r="J47" s="33" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="K47" s="33" t="n">
-        <v>0</v>
+        <v>2233</v>
       </c>
       <c r="L47" s="33" t="n">
-        <v>75.3</v>
+        <v>64.3</v>
       </c>
       <c r="M47" s="33" t="n">
-        <v>14974</v>
+        <v>113222</v>
       </c>
       <c r="N47" s="34" t="inlineStr">
         <is>
@@ -13344,7 +13344,7 @@
         <v>0.6662489019033675</v>
       </c>
       <c r="CD47" s="49" t="n">
-        <v>1.000013624847218</v>
+        <v>0.1129237126553488</v>
       </c>
     </row>
     <row r="48">
@@ -13359,37 +13359,37 @@
         </is>
       </c>
       <c r="C48" s="33" t="n">
-        <v>494</v>
+        <v>39025</v>
       </c>
       <c r="D48" s="33" t="n">
-        <v>0.6</v>
+        <v>27.1</v>
       </c>
       <c r="E48" s="33" t="n">
-        <v>3</v>
+        <v>10591</v>
       </c>
       <c r="F48" s="33" t="n">
-        <v>98.90000000000001</v>
+        <v>65</v>
       </c>
       <c r="G48" s="33" t="n">
-        <v>489</v>
+        <v>25376</v>
       </c>
       <c r="H48" s="33" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="I48" s="33" t="n">
-        <v>0</v>
+        <v>655</v>
       </c>
       <c r="J48" s="33" t="n">
-        <v>0.6</v>
+        <v>6.2</v>
       </c>
       <c r="K48" s="33" t="n">
-        <v>3</v>
+        <v>2404</v>
       </c>
       <c r="L48" s="33" t="n">
-        <v>99.40000000000001</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="M48" s="33" t="n">
-        <v>491</v>
+        <v>28435</v>
       </c>
       <c r="N48" s="34" t="inlineStr">
         <is>
@@ -13606,7 +13606,7 @@
         <v>0.02155036538185987</v>
       </c>
       <c r="CD48" s="49" t="n">
-        <v>1.0000338992991</v>
+        <v>0.01265898132616927</v>
       </c>
     </row>
     <row r="49">
@@ -13621,37 +13621,37 @@
         </is>
       </c>
       <c r="C49" s="33" t="n">
-        <v>9197</v>
+        <v>36097</v>
       </c>
       <c r="D49" s="33" t="n">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="E49" s="33" t="n">
-        <v>363</v>
+        <v>1802</v>
       </c>
       <c r="F49" s="33" t="n">
-        <v>90.90000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="G49" s="33" t="n">
-        <v>8358</v>
+        <v>32454</v>
       </c>
       <c r="H49" s="33" t="n">
-        <v>4.4</v>
+        <v>1.3</v>
       </c>
       <c r="I49" s="33" t="n">
-        <v>401</v>
+        <v>476</v>
       </c>
       <c r="J49" s="33" t="n">
-        <v>0.8</v>
+        <v>3.8</v>
       </c>
       <c r="K49" s="33" t="n">
-        <v>76</v>
+        <v>1364</v>
       </c>
       <c r="L49" s="33" t="n">
-        <v>96.09999999999999</v>
+        <v>95</v>
       </c>
       <c r="M49" s="33" t="n">
-        <v>8835</v>
+        <v>34295</v>
       </c>
       <c r="N49" s="34" t="inlineStr">
         <is>
@@ -13868,7 +13868,7 @@
         <v>0.06797081325383213</v>
       </c>
       <c r="CD49" s="49" t="n">
-        <v>1.000049444457492</v>
+        <v>0.2547983140060269</v>
       </c>
     </row>
     <row r="50">
@@ -13883,37 +13883,37 @@
         </is>
       </c>
       <c r="C50" s="33" t="n">
-        <v>6215</v>
+        <v>30823</v>
       </c>
       <c r="D50" s="33" t="n">
-        <v>16.5</v>
+        <v>47.6</v>
       </c>
       <c r="E50" s="33" t="n">
-        <v>1026</v>
+        <v>14674</v>
       </c>
       <c r="F50" s="33" t="n">
-        <v>74.90000000000001</v>
+        <v>47.2</v>
       </c>
       <c r="G50" s="33" t="n">
-        <v>4656</v>
+        <v>14556</v>
       </c>
       <c r="H50" s="33" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="I50" s="33" t="n">
-        <v>39</v>
+        <v>393</v>
       </c>
       <c r="J50" s="33" t="n">
-        <v>7.9</v>
+        <v>3.9</v>
       </c>
       <c r="K50" s="33" t="n">
-        <v>493</v>
+        <v>1200</v>
       </c>
       <c r="L50" s="33" t="n">
-        <v>83.5</v>
+        <v>52.4</v>
       </c>
       <c r="M50" s="33" t="n">
-        <v>5189</v>
+        <v>16150</v>
       </c>
       <c r="N50" s="34" t="inlineStr">
         <is>
@@ -14130,7 +14130,7 @@
         <v>0.4592630278363253</v>
       </c>
       <c r="CD50" s="49" t="n">
-        <v>1.000017194673616</v>
+        <v>0.2016386096387932</v>
       </c>
     </row>
     <row r="51">
@@ -14715,19 +14715,19 @@
         </is>
       </c>
       <c r="C53" s="33" t="n">
-        <v>3184</v>
+        <v>17438</v>
       </c>
       <c r="D53" s="33" t="n">
-        <v>48.5</v>
+        <v>54.4</v>
       </c>
       <c r="E53" s="33" t="n">
-        <v>1545</v>
+        <v>9492</v>
       </c>
       <c r="F53" s="33" t="n">
-        <v>51.5</v>
+        <v>45.6</v>
       </c>
       <c r="G53" s="33" t="n">
-        <v>1639</v>
+        <v>7945</v>
       </c>
       <c r="H53" s="33" t="n">
         <v>0</v>
@@ -14742,10 +14742,10 @@
         <v>0</v>
       </c>
       <c r="L53" s="33" t="n">
-        <v>51.5</v>
+        <v>45.6</v>
       </c>
       <c r="M53" s="33" t="n">
-        <v>1639</v>
+        <v>7945</v>
       </c>
       <c r="N53" s="34" t="inlineStr">
         <is>
@@ -14962,7 +14962,7 @@
         <v>0.2460812539987204</v>
       </c>
       <c r="CD53" s="49" t="n">
-        <v>0.999928503432941</v>
+        <v>0.1825766919905083</v>
       </c>
     </row>
     <row r="54">
@@ -15547,37 +15547,37 @@
         </is>
       </c>
       <c r="C56" s="33" t="n">
-        <v>11328</v>
+        <v>37431</v>
       </c>
       <c r="D56" s="33" t="n">
-        <v>25.6</v>
+        <v>37.3</v>
       </c>
       <c r="E56" s="33" t="n">
-        <v>2901</v>
+        <v>13979</v>
       </c>
       <c r="F56" s="33" t="n">
-        <v>64.59999999999999</v>
+        <v>56.6</v>
       </c>
       <c r="G56" s="33" t="n">
-        <v>7322</v>
+        <v>21201</v>
       </c>
       <c r="H56" s="33" t="n">
-        <v>8.5</v>
+        <v>4.3</v>
       </c>
       <c r="I56" s="33" t="n">
-        <v>967</v>
+        <v>1604</v>
       </c>
       <c r="J56" s="33" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="K56" s="33" t="n">
-        <v>138</v>
+        <v>647</v>
       </c>
       <c r="L56" s="33" t="n">
-        <v>74.40000000000001</v>
+        <v>62.7</v>
       </c>
       <c r="M56" s="33" t="n">
-        <v>8427</v>
+        <v>23452</v>
       </c>
       <c r="N56" s="34" t="inlineStr">
         <is>
@@ -15794,7 +15794,7 @@
         <v>0.5462396107845124</v>
       </c>
       <c r="CD56" s="49" t="n">
-        <v>1.000002989127316</v>
+        <v>0.3026377564274061</v>
       </c>
     </row>
     <row r="57">
@@ -15809,37 +15809,37 @@
         </is>
       </c>
       <c r="C57" s="33" t="n">
-        <v>13858</v>
+        <v>18703</v>
       </c>
       <c r="D57" s="33" t="n">
-        <v>3.1</v>
+        <v>6.9</v>
       </c>
       <c r="E57" s="33" t="n">
-        <v>428</v>
+        <v>1297</v>
       </c>
       <c r="F57" s="33" t="n">
-        <v>85.2</v>
+        <v>81.5</v>
       </c>
       <c r="G57" s="33" t="n">
-        <v>11805</v>
+        <v>15245</v>
       </c>
       <c r="H57" s="33" t="n">
-        <v>6.8</v>
+        <v>5.7</v>
       </c>
       <c r="I57" s="33" t="n">
-        <v>941</v>
+        <v>1070</v>
       </c>
       <c r="J57" s="33" t="n">
-        <v>4.9</v>
+        <v>5.8</v>
       </c>
       <c r="K57" s="33" t="n">
-        <v>684</v>
+        <v>1091</v>
       </c>
       <c r="L57" s="33" t="n">
-        <v>96.90000000000001</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="M57" s="33" t="n">
-        <v>13430</v>
+        <v>17406</v>
       </c>
       <c r="N57" s="34" t="inlineStr">
         <is>
@@ -16056,7 +16056,7 @@
         <v>0.3353127879594553</v>
       </c>
       <c r="CD57" s="49" t="n">
-        <v>1.000008713824762</v>
+        <v>0.7409571061425198</v>
       </c>
     </row>
     <row r="58">
@@ -16071,37 +16071,37 @@
         </is>
       </c>
       <c r="C58" s="33" t="n">
-        <v>316</v>
+        <v>9849</v>
       </c>
       <c r="D58" s="33" t="n">
-        <v>1.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E58" s="33" t="n">
-        <v>4</v>
+        <v>905</v>
       </c>
       <c r="F58" s="33" t="n">
-        <v>97.8</v>
+        <v>77.3</v>
       </c>
       <c r="G58" s="33" t="n">
-        <v>309</v>
+        <v>7613</v>
       </c>
       <c r="H58" s="33" t="n">
-        <v>1.1</v>
+        <v>12.1</v>
       </c>
       <c r="I58" s="33" t="n">
-        <v>4</v>
+        <v>1189</v>
       </c>
       <c r="J58" s="33" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="K58" s="33" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="L58" s="33" t="n">
-        <v>98.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="M58" s="33" t="n">
-        <v>313</v>
+        <v>8945</v>
       </c>
       <c r="N58" s="34" t="inlineStr">
         <is>
@@ -16318,7 +16318,7 @@
         <v>0.1123930391308528</v>
       </c>
       <c r="CD58" s="49" t="n">
-        <v>1.001397898107846</v>
+        <v>0.03212932640898357</v>
       </c>
     </row>
     <row r="59">
@@ -16333,41 +16333,41 @@
         </is>
       </c>
       <c r="C59" s="33" t="n">
-        <v>10210</v>
+        <v>40378</v>
       </c>
       <c r="D59" s="33" t="n">
-        <v>36.3</v>
+        <v>43.2</v>
       </c>
       <c r="E59" s="33" t="n">
-        <v>3707</v>
+        <v>17456</v>
       </c>
       <c r="F59" s="33" t="n">
-        <v>42.5</v>
+        <v>37.7</v>
       </c>
       <c r="G59" s="33" t="n">
-        <v>4335</v>
+        <v>15215</v>
       </c>
       <c r="H59" s="33" t="n">
-        <v>20.1</v>
+        <v>16.8</v>
       </c>
       <c r="I59" s="33" t="n">
-        <v>2053</v>
+        <v>6801</v>
       </c>
       <c r="J59" s="33" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="K59" s="33" t="n">
-        <v>114</v>
+        <v>905</v>
       </c>
       <c r="L59" s="33" t="n">
-        <v>63.7</v>
+        <v>56.8</v>
       </c>
       <c r="M59" s="33" t="n">
-        <v>6502</v>
+        <v>22922</v>
       </c>
       <c r="N59" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O59" s="35" t="n">
@@ -16580,7 +16580,7 @@
         <v>0</v>
       </c>
       <c r="CD59" s="49" t="n">
-        <v>0.9999532479437409</v>
+        <v>0.2528486468251422</v>
       </c>
     </row>
     <row r="60">
@@ -16595,37 +16595,37 @@
         </is>
       </c>
       <c r="C60" s="33" t="n">
-        <v>18724</v>
+        <v>23742</v>
       </c>
       <c r="D60" s="33" t="n">
-        <v>11.7</v>
+        <v>18.2</v>
       </c>
       <c r="E60" s="33" t="n">
-        <v>2182</v>
+        <v>4316</v>
       </c>
       <c r="F60" s="33" t="n">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G60" s="33" t="n">
-        <v>16288</v>
+        <v>18985</v>
       </c>
       <c r="H60" s="33" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="I60" s="33" t="n">
-        <v>254</v>
+        <v>428</v>
       </c>
       <c r="J60" s="33" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K60" s="33" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L60" s="33" t="n">
-        <v>88.3</v>
+        <v>81.8</v>
       </c>
       <c r="M60" s="33" t="n">
-        <v>16542</v>
+        <v>19427</v>
       </c>
       <c r="N60" s="34" t="inlineStr">
         <is>
@@ -16842,7 +16842,7 @@
         <v>0.4475268781134164</v>
       </c>
       <c r="CD60" s="49" t="n">
-        <v>0.9999890236766334</v>
+        <v>0.7886359396563594</v>
       </c>
     </row>
     <row r="61">

</xml_diff>